<commit_message>
Finished selecting parts for bom, changed resistor values for leds
</commit_message>
<xml_diff>
--- a/hardware/SGI_BOM_V1.1.xlsx
+++ b/hardware/SGI_BOM_V1.1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ashto\Dev\SeniorDesign_SwanGanz\hardware\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80ABB676-6DF2-4C60-804A-9A452DA2FD7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CCFF16A-C2B2-4BBF-93FD-97B6E7396972}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{4EE8D713-7B25-4092-B83F-8A696BC138B6}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="342" uniqueCount="184">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="484" uniqueCount="252">
   <si>
     <t>Reference</t>
   </si>
@@ -206,12 +206,6 @@
     <t>R2, R22, R23, R24, R29, R30, R31, R36, R37, R38, R47, R50, R52</t>
   </si>
   <si>
-    <t>R3</t>
-  </si>
-  <si>
-    <t>R4, R5, R8, R9, R12, R13, R16, R18, R20, R21, R27, R28, R34, R35, R49</t>
-  </si>
-  <si>
     <t>R7, R10, R11, R14 , R15</t>
   </si>
   <si>
@@ -254,15 +248,6 @@
     <t>200R</t>
   </si>
   <si>
-    <t>17.5k</t>
-  </si>
-  <si>
-    <t>2k</t>
-  </si>
-  <si>
-    <t>R41, R43, R44</t>
-  </si>
-  <si>
     <t>R42</t>
   </si>
   <si>
@@ -299,18 +284,12 @@
     <t>U1</t>
   </si>
   <si>
-    <t>LM2937ESX-3.3_NOPB</t>
-  </si>
-  <si>
     <t>LM4041CILPR</t>
   </si>
   <si>
     <t>OPA2350</t>
   </si>
   <si>
-    <t>MSPM0G3507QPMRQ1</t>
-  </si>
-  <si>
     <t>INA122P</t>
   </si>
   <si>
@@ -588,6 +567,231 @@
   </si>
   <si>
     <t>667-ERJ-3RBD2702V</t>
+  </si>
+  <si>
+    <t>RE0603DRE078K2L</t>
+  </si>
+  <si>
+    <t>603-RE0603DRE078K2L</t>
+  </si>
+  <si>
+    <t>ERJ-PB3D2000V</t>
+  </si>
+  <si>
+    <t>1/5W</t>
+  </si>
+  <si>
+    <t>667-ERJ-PB3D2000V</t>
+  </si>
+  <si>
+    <t>667-ERJ-PB3D1742V</t>
+  </si>
+  <si>
+    <t>17.4k</t>
+  </si>
+  <si>
+    <t>ERJ-PB3D1742V</t>
+  </si>
+  <si>
+    <t>R4</t>
+  </si>
+  <si>
+    <t>279-CRGCQ0603J1M0</t>
+  </si>
+  <si>
+    <t>TE Connectivity / Holsworthy</t>
+  </si>
+  <si>
+    <t>CRGCQ0603J1M0</t>
+  </si>
+  <si>
+    <t>ERJ-PB3B1003V</t>
+  </si>
+  <si>
+    <t>R5, R8, R9, R12, R13, R16, R18, R20, R21, R27, R28, R34, R35, R49</t>
+  </si>
+  <si>
+    <t>67-ERJ-PB3B1003V</t>
+  </si>
+  <si>
+    <t>660-RK73Z1JLTD</t>
+  </si>
+  <si>
+    <t>1A</t>
+  </si>
+  <si>
+    <t>3A</t>
+  </si>
+  <si>
+    <t>JUMP</t>
+  </si>
+  <si>
+    <t>KOA</t>
+  </si>
+  <si>
+    <t>RK73Z1JLTD</t>
+  </si>
+  <si>
+    <t>RMCF0603FT750R</t>
+  </si>
+  <si>
+    <t>SEI Stackpole</t>
+  </si>
+  <si>
+    <t>708-RMCF0603FT750R</t>
+  </si>
+  <si>
+    <t>RK73H1JTTD1912F</t>
+  </si>
+  <si>
+    <t>KOA Speer</t>
+  </si>
+  <si>
+    <t>660-RK73H1JTTD1912F</t>
+  </si>
+  <si>
+    <t>652-CR0603FX-1652ELF</t>
+  </si>
+  <si>
+    <t>Bourns</t>
+  </si>
+  <si>
+    <t>CR0603-FX-1652ELF</t>
+  </si>
+  <si>
+    <t>Adam Tech</t>
+  </si>
+  <si>
+    <t>Toggle</t>
+  </si>
+  <si>
+    <t>737-SW-T3-1A-A-A3-S1</t>
+  </si>
+  <si>
+    <t>DDPAK</t>
+  </si>
+  <si>
+    <t>500mA</t>
+  </si>
+  <si>
+    <t>926-LM2937ES-3.3NOPB</t>
+  </si>
+  <si>
+    <t>Linear Regulator</t>
+  </si>
+  <si>
+    <t>LM2937ES-3.3/NOPB</t>
+  </si>
+  <si>
+    <t>3.3V LDO</t>
+  </si>
+  <si>
+    <t>TO-92</t>
+  </si>
+  <si>
+    <t>595-LM4041CILPR</t>
+  </si>
+  <si>
+    <t>M0G3507QPMRQ1</t>
+  </si>
+  <si>
+    <t>64 LQFP</t>
+  </si>
+  <si>
+    <t>595-M0G3507QPMRQ1</t>
+  </si>
+  <si>
+    <t>595-INA122P</t>
+  </si>
+  <si>
+    <t>8 PDIP</t>
+  </si>
+  <si>
+    <t>895-FT232RNL-REEL</t>
+  </si>
+  <si>
+    <t>FT232RNL-REEL</t>
+  </si>
+  <si>
+    <t>FTDI</t>
+  </si>
+  <si>
+    <t>SSOP-28</t>
+  </si>
+  <si>
+    <t>595-TSC2046IPWR</t>
+  </si>
+  <si>
+    <t>TSSOP-16</t>
+  </si>
+  <si>
+    <t>Breakout</t>
+  </si>
+  <si>
+    <t>485-1590</t>
+  </si>
+  <si>
+    <t>8-PDIP</t>
+  </si>
+  <si>
+    <t>+-20ppm</t>
+  </si>
+  <si>
+    <t>40MHz</t>
+  </si>
+  <si>
+    <t>35Ohms</t>
+  </si>
+  <si>
+    <t>Crystal</t>
+  </si>
+  <si>
+    <t>815-M8AIG-40-12-2ZT3</t>
+  </si>
+  <si>
+    <t>SPKM.28.8.A</t>
+  </si>
+  <si>
+    <t>960-SPKM.28.8.A</t>
+  </si>
+  <si>
+    <t>Wire</t>
+  </si>
+  <si>
+    <t>500mW</t>
+  </si>
+  <si>
+    <t>28mm</t>
+  </si>
+  <si>
+    <t>1596</t>
+  </si>
+  <si>
+    <t>5" LCD</t>
+  </si>
+  <si>
+    <t>40Pin</t>
+  </si>
+  <si>
+    <t>485-1596</t>
+  </si>
+  <si>
+    <t>Order Qty</t>
+  </si>
+  <si>
+    <t>1.8k</t>
+  </si>
+  <si>
+    <t>R44</t>
+  </si>
+  <si>
+    <t>R3, R41, R43</t>
+  </si>
+  <si>
+    <t>CRCW06031K80JNEA</t>
+  </si>
+  <si>
+    <t>71-CRCW0603J-1.8K-E3</t>
   </si>
 </sst>
 </file>
@@ -617,27 +821,12 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -648,9 +837,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -985,12 +1174,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2DB84AFE-AA67-459F-9D96-757C0A5835DB}">
-  <dimension ref="A1:L50"/>
+  <dimension ref="A1:M51"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>105</v>
+        <v>98</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
@@ -999,34 +1188,37 @@
         <v>1</v>
       </c>
       <c r="D1" t="s">
+        <v>246</v>
+      </c>
+      <c r="E1" t="s">
         <v>2</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>3</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>4</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>5</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>6</v>
       </c>
-      <c r="J1" t="s">
-        <v>113</v>
-      </c>
       <c r="K1" t="s">
-        <v>118</v>
+        <v>106</v>
       </c>
       <c r="L1" t="s">
+        <v>111</v>
+      </c>
+      <c r="M1" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1036,35 +1228,35 @@
       <c r="C2">
         <v>20</v>
       </c>
-      <c r="D2" t="s">
-        <v>112</v>
-      </c>
       <c r="E2" t="s">
-        <v>112</v>
+        <v>105</v>
       </c>
       <c r="F2" t="s">
+        <v>105</v>
+      </c>
+      <c r="G2" t="s">
         <v>9</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="H2" s="5">
+      <c r="I2" s="4">
         <v>0.05</v>
       </c>
-      <c r="I2" t="s">
-        <v>115</v>
-      </c>
-      <c r="J2" s="5" t="s">
-        <v>114</v>
-      </c>
-      <c r="K2" t="s">
-        <v>132</v>
+      <c r="J2" t="s">
+        <v>108</v>
+      </c>
+      <c r="K2" s="4" t="s">
+        <v>107</v>
       </c>
       <c r="L2" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
+        <v>125</v>
+      </c>
+      <c r="M2" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1074,70 +1266,70 @@
       <c r="C3">
         <v>2</v>
       </c>
-      <c r="D3" t="s">
-        <v>129</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="F3" t="s">
-        <v>127</v>
-      </c>
-      <c r="G3" s="1" t="s">
+      <c r="E3" t="s">
+        <v>122</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="G3" t="s">
+        <v>120</v>
+      </c>
+      <c r="H3" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="H3" s="5">
+      <c r="I3" s="4">
         <v>0.05</v>
       </c>
-      <c r="I3" t="s">
-        <v>120</v>
-      </c>
       <c r="J3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="K3" t="s">
-        <v>131</v>
+        <v>107</v>
       </c>
       <c r="L3" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
+        <v>124</v>
+      </c>
+      <c r="M3" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>128</v>
+        <v>121</v>
       </c>
       <c r="C4">
         <v>4</v>
       </c>
-      <c r="D4" t="s">
-        <v>116</v>
-      </c>
       <c r="E4" t="s">
-        <v>117</v>
+        <v>109</v>
       </c>
       <c r="F4" t="s">
+        <v>110</v>
+      </c>
+      <c r="G4" t="s">
         <v>12</v>
       </c>
-      <c r="G4" s="1" t="s">
+      <c r="H4" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="H4" s="5">
+      <c r="I4" s="4">
         <v>0.1</v>
       </c>
-      <c r="I4" t="s">
-        <v>120</v>
-      </c>
       <c r="J4" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="K4" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
+        <v>107</v>
+      </c>
+      <c r="L4" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1147,35 +1339,35 @@
       <c r="C5">
         <v>1</v>
       </c>
-      <c r="D5" t="s">
-        <v>121</v>
-      </c>
       <c r="E5" t="s">
-        <v>122</v>
+        <v>114</v>
       </c>
       <c r="F5" t="s">
+        <v>115</v>
+      </c>
+      <c r="G5" t="s">
         <v>14</v>
       </c>
-      <c r="G5" s="1" t="s">
+      <c r="H5" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="H5" s="5">
+      <c r="I5" s="4">
         <v>0.05</v>
       </c>
-      <c r="I5" t="s">
-        <v>120</v>
-      </c>
       <c r="J5" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="K5" t="s">
-        <v>123</v>
+        <v>107</v>
       </c>
       <c r="L5" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
+        <v>116</v>
+      </c>
+      <c r="M5" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1185,35 +1377,35 @@
       <c r="C6">
         <v>1</v>
       </c>
-      <c r="D6" t="s">
-        <v>124</v>
-      </c>
       <c r="E6" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
       <c r="F6" t="s">
+        <v>118</v>
+      </c>
+      <c r="G6" t="s">
         <v>16</v>
       </c>
-      <c r="G6" s="1" t="s">
+      <c r="H6" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="H6" s="5">
+      <c r="I6" s="4">
         <v>0.1</v>
       </c>
-      <c r="I6" t="s">
-        <v>120</v>
-      </c>
       <c r="J6" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="K6" t="s">
-        <v>126</v>
+        <v>107</v>
       </c>
       <c r="L6" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
+        <v>119</v>
+      </c>
+      <c r="M6" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1223,35 +1415,35 @@
       <c r="C7">
         <v>2</v>
       </c>
-      <c r="D7" t="s">
-        <v>134</v>
-      </c>
       <c r="E7" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="F7" t="s">
+        <v>128</v>
+      </c>
+      <c r="G7" t="s">
         <v>18</v>
       </c>
-      <c r="G7" s="1" t="s">
+      <c r="H7" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="H7" s="5">
+      <c r="I7" s="4">
         <v>0.01</v>
       </c>
-      <c r="I7" t="s">
-        <v>136</v>
-      </c>
       <c r="J7" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="K7" t="s">
-        <v>137</v>
+        <v>126</v>
       </c>
       <c r="L7" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.35">
+        <v>130</v>
+      </c>
+      <c r="M7" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1261,35 +1453,35 @@
       <c r="C8">
         <v>1</v>
       </c>
-      <c r="D8" t="s">
-        <v>138</v>
-      </c>
       <c r="E8" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="F8" t="s">
+        <v>128</v>
+      </c>
+      <c r="G8" t="s">
         <v>20</v>
       </c>
-      <c r="G8" s="1" t="s">
+      <c r="H8" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="H8" s="5">
+      <c r="I8" s="4">
         <v>0.05</v>
       </c>
-      <c r="I8" t="s">
-        <v>115</v>
-      </c>
       <c r="J8" t="s">
-        <v>133</v>
+        <v>108</v>
       </c>
       <c r="K8" t="s">
-        <v>139</v>
+        <v>126</v>
       </c>
       <c r="L8" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
+        <v>132</v>
+      </c>
+      <c r="M8" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1299,32 +1491,32 @@
       <c r="C9">
         <v>1</v>
       </c>
-      <c r="D9" t="s">
-        <v>141</v>
-      </c>
-      <c r="F9" t="s">
+      <c r="E9" t="s">
+        <v>134</v>
+      </c>
+      <c r="G9" t="s">
         <v>22</v>
       </c>
-      <c r="G9" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="H9" s="5">
+      <c r="H9" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="I9" s="4">
         <v>0.1</v>
       </c>
-      <c r="I9" t="s">
-        <v>142</v>
-      </c>
       <c r="J9" t="s">
-        <v>114</v>
+        <v>135</v>
       </c>
       <c r="K9" t="s">
-        <v>143</v>
+        <v>107</v>
       </c>
       <c r="L9" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.35">
+        <v>136</v>
+      </c>
+      <c r="M9" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1334,35 +1526,35 @@
       <c r="C10">
         <v>1</v>
       </c>
-      <c r="D10" t="s">
-        <v>145</v>
-      </c>
       <c r="E10" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="F10" t="s">
-        <v>144</v>
-      </c>
-      <c r="G10" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="G10" t="s">
+        <v>137</v>
+      </c>
+      <c r="H10" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="H10" s="5">
+      <c r="I10" s="4">
         <v>0.1</v>
       </c>
-      <c r="I10" t="s">
-        <v>120</v>
-      </c>
       <c r="J10" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="K10" t="s">
-        <v>146</v>
+        <v>107</v>
       </c>
       <c r="L10" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
+        <v>139</v>
+      </c>
+      <c r="M10" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1372,21 +1564,18 @@
       <c r="C11">
         <v>2</v>
       </c>
-      <c r="D11" t="s">
-        <v>27</v>
-      </c>
       <c r="E11" t="s">
         <v>27</v>
       </c>
       <c r="F11" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G11" t="s">
+        <v>26</v>
+      </c>
+      <c r="H11" t="s">
         <v>25</v>
       </c>
-      <c r="H11" t="s">
-        <v>26</v>
-      </c>
       <c r="I11" t="s">
         <v>26</v>
       </c>
@@ -1397,10 +1586,13 @@
         <v>26</v>
       </c>
       <c r="L11" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.35">
+        <v>26</v>
+      </c>
+      <c r="M11" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1410,35 +1602,35 @@
       <c r="C12">
         <v>1</v>
       </c>
-      <c r="D12" t="s">
+      <c r="E12" t="s">
         <v>29</v>
       </c>
-      <c r="E12" t="s">
-        <v>147</v>
-      </c>
       <c r="F12" t="s">
-        <v>148</v>
-      </c>
-      <c r="G12" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="G12" t="s">
+        <v>141</v>
+      </c>
+      <c r="H12" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="H12" t="s">
-        <v>26</v>
-      </c>
       <c r="I12" t="s">
-        <v>149</v>
+        <v>26</v>
       </c>
       <c r="J12" t="s">
-        <v>150</v>
+        <v>142</v>
       </c>
       <c r="K12" t="s">
-        <v>151</v>
+        <v>143</v>
       </c>
       <c r="L12" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.35">
+        <v>144</v>
+      </c>
+      <c r="M12" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1448,35 +1640,35 @@
       <c r="C13">
         <v>1</v>
       </c>
-      <c r="D13" t="s">
+      <c r="E13" t="s">
         <v>30</v>
       </c>
-      <c r="E13" t="s">
-        <v>147</v>
-      </c>
       <c r="F13" t="s">
-        <v>153</v>
-      </c>
-      <c r="G13" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="G13" t="s">
+        <v>146</v>
+      </c>
+      <c r="H13" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="H13" t="s">
-        <v>26</v>
-      </c>
       <c r="I13" t="s">
-        <v>149</v>
+        <v>26</v>
       </c>
       <c r="J13" t="s">
-        <v>150</v>
+        <v>142</v>
       </c>
       <c r="K13" t="s">
-        <v>152</v>
+        <v>143</v>
       </c>
       <c r="L13" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.35">
+        <v>145</v>
+      </c>
+      <c r="M13" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1486,21 +1678,18 @@
       <c r="C14">
         <v>1</v>
       </c>
-      <c r="D14" t="s">
+      <c r="E14" t="s">
         <v>38</v>
       </c>
-      <c r="E14" t="s">
+      <c r="F14" t="s">
         <v>27</v>
       </c>
-      <c r="F14" t="s">
+      <c r="G14" t="s">
         <v>35</v>
       </c>
-      <c r="G14" t="s">
+      <c r="H14" t="s">
         <v>34</v>
       </c>
-      <c r="H14" t="s">
-        <v>26</v>
-      </c>
       <c r="I14" t="s">
         <v>26</v>
       </c>
@@ -1511,10 +1700,13 @@
         <v>26</v>
       </c>
       <c r="L14" t="s">
+        <v>26</v>
+      </c>
+      <c r="M14" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>14</v>
       </c>
@@ -1524,9 +1716,6 @@
       <c r="C15">
         <v>2</v>
       </c>
-      <c r="D15" t="s">
-        <v>26</v>
-      </c>
       <c r="E15" t="s">
         <v>26</v>
       </c>
@@ -1549,10 +1738,13 @@
         <v>26</v>
       </c>
       <c r="L15" t="s">
+        <v>26</v>
+      </c>
+      <c r="M15" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>15</v>
       </c>
@@ -1562,21 +1754,18 @@
       <c r="C16">
         <v>2</v>
       </c>
-      <c r="D16" t="s">
+      <c r="E16" t="s">
         <v>39</v>
       </c>
-      <c r="E16" t="s">
+      <c r="F16" t="s">
         <v>27</v>
       </c>
-      <c r="F16" t="s">
+      <c r="G16" t="s">
         <v>40</v>
       </c>
-      <c r="G16" t="s">
+      <c r="H16" t="s">
         <v>34</v>
       </c>
-      <c r="H16" t="s">
-        <v>26</v>
-      </c>
       <c r="I16" t="s">
         <v>26</v>
       </c>
@@ -1587,10 +1776,13 @@
         <v>26</v>
       </c>
       <c r="L16" t="s">
+        <v>26</v>
+      </c>
+      <c r="M16" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>16</v>
       </c>
@@ -1600,21 +1792,18 @@
       <c r="C17">
         <v>2</v>
       </c>
-      <c r="D17" t="s">
+      <c r="E17" t="s">
         <v>38</v>
       </c>
-      <c r="E17" t="s">
+      <c r="F17" t="s">
         <v>42</v>
       </c>
-      <c r="F17" t="s">
+      <c r="G17" t="s">
         <v>40</v>
       </c>
-      <c r="G17" t="s">
+      <c r="H17" t="s">
         <v>34</v>
       </c>
-      <c r="H17" t="s">
-        <v>26</v>
-      </c>
       <c r="I17" t="s">
         <v>26</v>
       </c>
@@ -1625,10 +1814,13 @@
         <v>26</v>
       </c>
       <c r="L17" t="s">
+        <v>26</v>
+      </c>
+      <c r="M17" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>17</v>
       </c>
@@ -1638,21 +1830,18 @@
       <c r="C18">
         <v>1</v>
       </c>
-      <c r="D18" t="s">
+      <c r="E18" t="s">
         <v>38</v>
       </c>
-      <c r="E18" t="s">
+      <c r="F18" t="s">
         <v>27</v>
       </c>
-      <c r="F18" t="s">
+      <c r="G18" t="s">
         <v>44</v>
       </c>
-      <c r="G18" t="s">
+      <c r="H18" t="s">
         <v>34</v>
       </c>
-      <c r="H18" t="s">
-        <v>26</v>
-      </c>
       <c r="I18" t="s">
         <v>26</v>
       </c>
@@ -1663,10 +1852,13 @@
         <v>26</v>
       </c>
       <c r="L18" t="s">
+        <v>26</v>
+      </c>
+      <c r="M18" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>18</v>
       </c>
@@ -1676,21 +1868,18 @@
       <c r="C19">
         <v>1</v>
       </c>
-      <c r="D19" t="s">
+      <c r="E19" t="s">
         <v>38</v>
       </c>
-      <c r="E19" t="s">
+      <c r="F19" t="s">
         <v>27</v>
       </c>
-      <c r="F19" t="s">
+      <c r="G19" t="s">
         <v>46</v>
       </c>
-      <c r="G19" t="s">
+      <c r="H19" t="s">
         <v>34</v>
       </c>
-      <c r="H19" t="s">
-        <v>26</v>
-      </c>
       <c r="I19" t="s">
         <v>26</v>
       </c>
@@ -1701,10 +1890,13 @@
         <v>26</v>
       </c>
       <c r="L19" t="s">
+        <v>26</v>
+      </c>
+      <c r="M19" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>19</v>
       </c>
@@ -1714,73 +1906,73 @@
       <c r="C20">
         <v>1</v>
       </c>
-      <c r="D20">
+      <c r="E20">
         <v>1935161</v>
       </c>
-      <c r="E20" t="s">
-        <v>158</v>
-      </c>
       <c r="F20" t="s">
-        <v>159</v>
+        <v>151</v>
       </c>
       <c r="G20" t="s">
-        <v>160</v>
+        <v>152</v>
       </c>
       <c r="H20" t="s">
-        <v>26</v>
+        <v>153</v>
       </c>
       <c r="I20" t="s">
-        <v>161</v>
+        <v>26</v>
       </c>
       <c r="J20" t="s">
+        <v>154</v>
+      </c>
+      <c r="K20" t="s">
         <v>48</v>
       </c>
-      <c r="K20" t="s">
-        <v>162</v>
-      </c>
       <c r="L20" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.35">
+        <v>155</v>
+      </c>
+      <c r="M20" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>165</v>
+        <v>158</v>
       </c>
       <c r="C21">
         <v>1</v>
       </c>
-      <c r="D21" t="s">
+      <c r="E21" t="s">
         <v>51</v>
       </c>
-      <c r="E21" t="s">
-        <v>166</v>
-      </c>
       <c r="F21" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
       <c r="G21" t="s">
-        <v>106</v>
+        <v>160</v>
       </c>
       <c r="H21" t="s">
-        <v>26</v>
+        <v>99</v>
       </c>
       <c r="I21" t="s">
-        <v>164</v>
+        <v>26</v>
       </c>
       <c r="J21" t="s">
+        <v>157</v>
+      </c>
+      <c r="K21" t="s">
         <v>52</v>
       </c>
-      <c r="K21" t="s">
-        <v>163</v>
-      </c>
       <c r="L21" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.35">
+        <v>156</v>
+      </c>
+      <c r="M21" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A22">
         <v>21</v>
       </c>
@@ -1790,35 +1982,35 @@
       <c r="C22">
         <v>2</v>
       </c>
-      <c r="D22" t="s">
-        <v>168</v>
-      </c>
       <c r="E22" t="s">
-        <v>122</v>
+        <v>161</v>
       </c>
       <c r="F22" t="s">
+        <v>115</v>
+      </c>
+      <c r="G22" t="s">
         <v>54</v>
       </c>
-      <c r="G22" s="1" t="s">
+      <c r="H22" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="H22" s="4">
+      <c r="I22" s="3">
         <v>5.0000000000000001E-3</v>
       </c>
-      <c r="I22" t="s">
-        <v>169</v>
-      </c>
       <c r="J22" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="K22" t="s">
-        <v>171</v>
+        <v>163</v>
       </c>
       <c r="L22" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.35">
+        <v>164</v>
+      </c>
+      <c r="M22" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A23">
         <v>22</v>
       </c>
@@ -1828,407 +2020,584 @@
       <c r="C23">
         <v>13</v>
       </c>
-      <c r="D23" t="s">
-        <v>172</v>
-      </c>
       <c r="E23" t="s">
-        <v>122</v>
+        <v>165</v>
       </c>
       <c r="F23" t="s">
-        <v>65</v>
-      </c>
-      <c r="G23" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="G23" t="s">
+        <v>63</v>
+      </c>
+      <c r="H23" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="H23" s="4">
+      <c r="I23" s="3">
         <v>5.0000000000000001E-3</v>
       </c>
-      <c r="I23" t="s">
-        <v>169</v>
-      </c>
       <c r="J23" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="K23" t="s">
-        <v>173</v>
+        <v>163</v>
       </c>
       <c r="L23" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.35">
+        <v>166</v>
+      </c>
+      <c r="M23" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A24">
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>56</v>
+        <v>249</v>
       </c>
       <c r="C24">
-        <v>1</v>
-      </c>
-      <c r="D24" t="s">
-        <v>174</v>
+        <v>3</v>
       </c>
       <c r="E24" t="s">
-        <v>122</v>
+        <v>167</v>
       </c>
       <c r="F24" t="s">
-        <v>66</v>
-      </c>
-      <c r="G24" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="G24" t="s">
+        <v>64</v>
+      </c>
+      <c r="H24" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="H24" s="4">
+      <c r="I24" s="3">
         <v>5.0000000000000001E-3</v>
       </c>
-      <c r="I24" t="s">
-        <v>169</v>
-      </c>
       <c r="J24" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="K24" t="s">
-        <v>175</v>
+        <v>163</v>
       </c>
       <c r="L24" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.35">
+        <v>168</v>
+      </c>
+      <c r="M24" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A25">
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>57</v>
+        <v>185</v>
       </c>
       <c r="C25">
-        <v>15</v>
-      </c>
-      <c r="D25" t="s">
-        <v>177</v>
+        <v>1</v>
       </c>
       <c r="E25" t="s">
-        <v>122</v>
+        <v>189</v>
       </c>
       <c r="F25" t="s">
-        <v>67</v>
-      </c>
-      <c r="G25" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="G25" t="s">
+        <v>65</v>
+      </c>
+      <c r="H25" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="H25" s="4">
-        <v>5.0000000000000001E-3</v>
-      </c>
-      <c r="I25" t="s">
-        <v>169</v>
+      <c r="I25" s="3">
+        <v>1E-3</v>
       </c>
       <c r="J25" t="s">
-        <v>170</v>
+        <v>180</v>
       </c>
       <c r="K25" t="s">
-        <v>176</v>
+        <v>163</v>
       </c>
       <c r="L25" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.35">
+        <v>191</v>
+      </c>
+      <c r="M25" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A26">
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>58</v>
+        <v>190</v>
       </c>
       <c r="C26">
+        <v>15</v>
+      </c>
+      <c r="E26" t="s">
+        <v>170</v>
+      </c>
+      <c r="F26" t="s">
+        <v>115</v>
+      </c>
+      <c r="G26" t="s">
+        <v>65</v>
+      </c>
+      <c r="H26" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="I26" s="3">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="J26" t="s">
+        <v>162</v>
+      </c>
+      <c r="K26" t="s">
+        <v>163</v>
+      </c>
+      <c r="L26" t="s">
+        <v>169</v>
+      </c>
+      <c r="M26" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A27">
+        <v>26</v>
+      </c>
+      <c r="B27" t="s">
+        <v>56</v>
+      </c>
+      <c r="C27">
         <v>5</v>
       </c>
-      <c r="D26" t="s">
-        <v>178</v>
-      </c>
-      <c r="E26" t="s">
-        <v>166</v>
-      </c>
-      <c r="F26" t="s">
-        <v>68</v>
-      </c>
-      <c r="G26" s="1" t="s">
+      <c r="E27" t="s">
+        <v>171</v>
+      </c>
+      <c r="F27" t="s">
+        <v>159</v>
+      </c>
+      <c r="G27" t="s">
+        <v>66</v>
+      </c>
+      <c r="H27" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="H26" s="5">
+      <c r="I27" s="4">
         <v>0.01</v>
       </c>
-      <c r="I26" t="s">
-        <v>179</v>
-      </c>
-      <c r="J26" t="s">
-        <v>170</v>
-      </c>
-      <c r="K26" t="s">
-        <v>180</v>
-      </c>
-      <c r="L26" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A27">
-        <v>26</v>
-      </c>
-      <c r="B27" t="s">
-        <v>59</v>
-      </c>
-      <c r="C27">
-        <v>2</v>
-      </c>
-      <c r="D27" t="s">
-        <v>181</v>
-      </c>
-      <c r="E27" t="s">
-        <v>182</v>
-      </c>
-      <c r="F27" t="s">
-        <v>69</v>
-      </c>
-      <c r="G27" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="H27" s="4">
-        <v>5.0000000000000001E-3</v>
-      </c>
-      <c r="I27" t="s">
-        <v>169</v>
-      </c>
       <c r="J27" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="K27" t="s">
-        <v>183</v>
+        <v>163</v>
       </c>
       <c r="L27" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.35">
+        <v>173</v>
+      </c>
+      <c r="M27" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A28">
         <v>27</v>
       </c>
       <c r="B28" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="C28">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="E28" t="s">
+        <v>174</v>
       </c>
       <c r="F28" t="s">
-        <v>70</v>
-      </c>
-      <c r="G28" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="G28" t="s">
+        <v>67</v>
+      </c>
+      <c r="H28" s="1" t="s">
         <v>10</v>
       </c>
+      <c r="I28" s="3">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="J28" t="s">
+        <v>162</v>
+      </c>
+      <c r="K28" t="s">
+        <v>163</v>
+      </c>
       <c r="L28" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.35">
+        <v>176</v>
+      </c>
+      <c r="M28" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A29">
         <v>28</v>
       </c>
       <c r="B29" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="C29">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="E29" t="s">
+        <v>177</v>
       </c>
       <c r="F29" t="s">
-        <v>71</v>
-      </c>
-      <c r="G29" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="G29" t="s">
+        <v>68</v>
+      </c>
+      <c r="H29" s="1" t="s">
         <v>10</v>
       </c>
+      <c r="I29" s="3">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="J29" t="s">
+        <v>162</v>
+      </c>
+      <c r="K29" t="s">
+        <v>163</v>
+      </c>
       <c r="L29" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.35">
+        <v>178</v>
+      </c>
+      <c r="M29" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A30">
         <v>29</v>
       </c>
       <c r="B30" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C30">
         <v>2</v>
       </c>
+      <c r="E30" t="s">
+        <v>179</v>
+      </c>
       <c r="F30" t="s">
-        <v>72</v>
-      </c>
-      <c r="G30" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="G30" t="s">
+        <v>69</v>
+      </c>
+      <c r="H30" s="1" t="s">
         <v>10</v>
       </c>
+      <c r="I30" s="3">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="J30" t="s">
+        <v>180</v>
+      </c>
+      <c r="K30" t="s">
+        <v>163</v>
+      </c>
       <c r="L30" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.35">
+        <v>181</v>
+      </c>
+      <c r="M30" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="31" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A31">
         <v>30</v>
       </c>
       <c r="B31" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="C31">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="E31" t="s">
+        <v>184</v>
       </c>
       <c r="F31" t="s">
-        <v>64</v>
-      </c>
-      <c r="G31" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="G31" t="s">
+        <v>183</v>
+      </c>
+      <c r="H31" s="1" t="s">
         <v>10</v>
       </c>
+      <c r="I31" s="3">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="J31" t="s">
+        <v>180</v>
+      </c>
+      <c r="K31" t="s">
+        <v>163</v>
+      </c>
       <c r="L31" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.35">
+        <v>182</v>
+      </c>
+      <c r="M31" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="32" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A32">
         <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>74</v>
+        <v>61</v>
       </c>
       <c r="C32">
-        <v>3</v>
-      </c>
-      <c r="F32" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="G32" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E32" t="s">
+        <v>188</v>
+      </c>
+      <c r="F32" t="s">
+        <v>187</v>
+      </c>
+      <c r="G32" t="s">
+        <v>62</v>
+      </c>
+      <c r="H32" s="1" t="s">
         <v>10</v>
       </c>
+      <c r="I32" s="4">
+        <v>0.05</v>
+      </c>
+      <c r="J32" t="s">
+        <v>162</v>
+      </c>
+      <c r="K32" t="s">
+        <v>163</v>
+      </c>
       <c r="L32" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.35">
+        <v>186</v>
+      </c>
+      <c r="M32" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="33" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A33">
         <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>75</v>
+        <v>248</v>
       </c>
       <c r="C33">
         <v>1</v>
       </c>
+      <c r="E33" t="s">
+        <v>250</v>
+      </c>
       <c r="F33" t="s">
-        <v>107</v>
-      </c>
-      <c r="G33" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="G33" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="H33" s="1" t="s">
         <v>10</v>
       </c>
+      <c r="I33" s="4">
+        <v>0.05</v>
+      </c>
+      <c r="J33" t="s">
+        <v>172</v>
+      </c>
+      <c r="K33" t="s">
+        <v>163</v>
+      </c>
       <c r="L33" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.35">
+        <v>251</v>
+      </c>
+      <c r="M33" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="34" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A34">
         <v>33</v>
       </c>
       <c r="B34" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="C34">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="E34" t="s">
+        <v>197</v>
       </c>
       <c r="F34" t="s">
-        <v>77</v>
-      </c>
-      <c r="G34" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="G34" t="s">
+        <v>100</v>
+      </c>
+      <c r="H34" s="1" t="s">
         <v>10</v>
       </c>
+      <c r="I34" t="s">
+        <v>195</v>
+      </c>
+      <c r="J34" t="s">
+        <v>193</v>
+      </c>
+      <c r="K34" t="s">
+        <v>163</v>
+      </c>
       <c r="L34" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.35">
+        <v>192</v>
+      </c>
+      <c r="M34" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="35" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A35">
         <v>34</v>
       </c>
       <c r="B35" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
       <c r="C35">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="E35" t="s">
+        <v>198</v>
       </c>
       <c r="F35" t="s">
-        <v>78</v>
-      </c>
-      <c r="G35" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="G35" t="s">
+        <v>72</v>
+      </c>
+      <c r="H35" s="1" t="s">
         <v>10</v>
       </c>
+      <c r="I35" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="J35" t="s">
+        <v>162</v>
+      </c>
+      <c r="K35" t="s">
+        <v>163</v>
+      </c>
       <c r="L35" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.35">
+        <v>200</v>
+      </c>
+      <c r="M35" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="36" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A36">
         <v>35</v>
       </c>
       <c r="B36" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="C36">
         <v>1</v>
       </c>
+      <c r="E36" t="s">
+        <v>201</v>
+      </c>
       <c r="F36" t="s">
-        <v>81</v>
-      </c>
-      <c r="G36" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="G36" t="s">
+        <v>73</v>
+      </c>
+      <c r="H36" s="1" t="s">
         <v>10</v>
       </c>
+      <c r="I36" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="J36" t="s">
+        <v>162</v>
+      </c>
+      <c r="K36" t="s">
+        <v>163</v>
+      </c>
       <c r="L36" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.35">
+        <v>203</v>
+      </c>
+      <c r="M36" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="37" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A37">
         <v>36</v>
       </c>
       <c r="B37" t="s">
-        <v>83</v>
+        <v>75</v>
       </c>
       <c r="C37">
         <v>1</v>
       </c>
+      <c r="E37" t="s">
+        <v>206</v>
+      </c>
       <c r="F37" t="s">
-        <v>82</v>
+        <v>205</v>
       </c>
       <c r="G37" t="s">
-        <v>26</v>
+        <v>76</v>
+      </c>
+      <c r="H37" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="I37" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="J37" t="s">
+        <v>162</v>
+      </c>
+      <c r="K37" t="s">
+        <v>163</v>
       </c>
       <c r="L37" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.35">
+        <v>204</v>
+      </c>
+      <c r="M37" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="38" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A38">
         <v>37</v>
       </c>
       <c r="B38" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="C38">
-        <v>5</v>
-      </c>
-      <c r="D38" t="s">
-        <v>27</v>
+        <v>1</v>
       </c>
       <c r="E38" t="s">
-        <v>27</v>
+        <v>77</v>
       </c>
       <c r="F38" t="s">
-        <v>26</v>
+        <v>207</v>
       </c>
       <c r="G38" t="s">
-        <v>26</v>
+        <v>77</v>
       </c>
       <c r="H38" t="s">
         <v>26</v>
@@ -2236,224 +2605,520 @@
       <c r="I38" t="s">
         <v>26</v>
       </c>
+      <c r="J38" t="s">
+        <v>194</v>
+      </c>
+      <c r="K38" t="s">
+        <v>208</v>
+      </c>
       <c r="L38" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.35">
+        <v>209</v>
+      </c>
+      <c r="M38" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="39" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A39">
         <v>38</v>
       </c>
       <c r="B39" t="s">
-        <v>86</v>
+        <v>79</v>
       </c>
       <c r="C39">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E39" t="s">
-        <v>108</v>
+        <v>27</v>
       </c>
       <c r="F39" t="s">
-        <v>87</v>
+        <v>27</v>
+      </c>
+      <c r="G39" t="s">
+        <v>26</v>
+      </c>
+      <c r="H39" t="s">
+        <v>26</v>
+      </c>
+      <c r="I39" t="s">
+        <v>26</v>
+      </c>
+      <c r="J39" t="s">
+        <v>26</v>
+      </c>
+      <c r="K39" t="s">
+        <v>26</v>
       </c>
       <c r="L39" t="s">
+        <v>26</v>
+      </c>
+      <c r="M39" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A40">
         <v>39</v>
       </c>
       <c r="B40" t="s">
-        <v>96</v>
+        <v>81</v>
       </c>
       <c r="C40">
         <v>1</v>
       </c>
       <c r="E40" t="s">
-        <v>108</v>
+        <v>214</v>
       </c>
       <c r="F40" t="s">
-        <v>88</v>
+        <v>101</v>
+      </c>
+      <c r="G40" t="s">
+        <v>215</v>
+      </c>
+      <c r="H40" t="s">
+        <v>210</v>
+      </c>
+      <c r="I40" t="s">
+        <v>26</v>
+      </c>
+      <c r="J40" t="s">
+        <v>211</v>
+      </c>
+      <c r="K40" t="s">
+        <v>213</v>
       </c>
       <c r="L40" t="s">
+        <v>212</v>
+      </c>
+      <c r="M40" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A41">
         <v>40</v>
       </c>
       <c r="B41" t="s">
-        <v>97</v>
+        <v>89</v>
       </c>
       <c r="C41">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E41" t="s">
-        <v>108</v>
+        <v>82</v>
       </c>
       <c r="F41" t="s">
-        <v>89</v>
+        <v>101</v>
+      </c>
+      <c r="G41" t="s">
+        <v>82</v>
+      </c>
+      <c r="H41" t="s">
+        <v>216</v>
+      </c>
+      <c r="I41" t="s">
+        <v>26</v>
+      </c>
+      <c r="J41" t="s">
+        <v>26</v>
+      </c>
+      <c r="K41" t="s">
+        <v>26</v>
       </c>
       <c r="L41" t="s">
+        <v>217</v>
+      </c>
+      <c r="M41" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A42">
         <v>41</v>
       </c>
       <c r="B42" t="s">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="C42">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E42" t="s">
-        <v>108</v>
+        <v>83</v>
       </c>
       <c r="F42" t="s">
-        <v>90</v>
+        <v>101</v>
+      </c>
+      <c r="G42" t="s">
+        <v>83</v>
+      </c>
+      <c r="H42" t="s">
+        <v>222</v>
+      </c>
+      <c r="I42" t="s">
+        <v>26</v>
+      </c>
+      <c r="J42" t="s">
+        <v>26</v>
+      </c>
+      <c r="K42" t="s">
+        <v>26</v>
       </c>
       <c r="L42" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.35">
+        <v>26</v>
+      </c>
+      <c r="M42" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="43" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A43">
         <v>42</v>
       </c>
       <c r="B43" t="s">
-        <v>99</v>
+        <v>91</v>
       </c>
       <c r="C43">
-        <v>3</v>
+        <v>1</v>
+      </c>
+      <c r="E43" t="s">
+        <v>218</v>
       </c>
       <c r="F43" t="s">
-        <v>91</v>
+        <v>101</v>
+      </c>
+      <c r="G43" t="s">
+        <v>26</v>
+      </c>
+      <c r="H43" t="s">
+        <v>219</v>
+      </c>
+      <c r="I43" t="s">
+        <v>26</v>
+      </c>
+      <c r="J43" t="s">
+        <v>26</v>
+      </c>
+      <c r="K43" t="s">
+        <v>26</v>
       </c>
       <c r="L43" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.35">
+        <v>220</v>
+      </c>
+      <c r="M43" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="44" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A44">
         <v>43</v>
       </c>
       <c r="B44" t="s">
-        <v>100</v>
+        <v>92</v>
       </c>
       <c r="C44">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="E44" t="s">
+        <v>84</v>
       </c>
       <c r="F44" t="s">
-        <v>92</v>
+        <v>101</v>
+      </c>
+      <c r="G44" t="s">
+        <v>84</v>
+      </c>
+      <c r="H44" t="s">
+        <v>222</v>
+      </c>
+      <c r="I44" t="s">
+        <v>26</v>
+      </c>
+      <c r="J44" t="s">
+        <v>26</v>
+      </c>
+      <c r="K44" t="s">
+        <v>26</v>
       </c>
       <c r="L44" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.35">
+        <v>221</v>
+      </c>
+      <c r="M44" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="45" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A45">
         <v>44</v>
       </c>
       <c r="B45" t="s">
-        <v>101</v>
+        <v>93</v>
       </c>
       <c r="C45">
         <v>1</v>
       </c>
+      <c r="E45" t="s">
+        <v>224</v>
+      </c>
       <c r="F45" t="s">
-        <v>93</v>
+        <v>225</v>
+      </c>
+      <c r="G45" t="s">
+        <v>85</v>
+      </c>
+      <c r="H45" t="s">
+        <v>226</v>
+      </c>
+      <c r="I45" t="s">
+        <v>26</v>
+      </c>
+      <c r="J45" t="s">
+        <v>26</v>
+      </c>
+      <c r="K45" t="s">
+        <v>26</v>
       </c>
       <c r="L45" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.35">
+        <v>223</v>
+      </c>
+      <c r="M45" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="46" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A46">
         <v>45</v>
       </c>
       <c r="B46" t="s">
-        <v>102</v>
+        <v>94</v>
       </c>
       <c r="C46">
         <v>1</v>
       </c>
       <c r="E46" t="s">
-        <v>156</v>
-      </c>
-      <c r="F46">
-        <v>1590</v>
+        <v>86</v>
+      </c>
+      <c r="F46" t="s">
+        <v>101</v>
+      </c>
+      <c r="G46" t="s">
+        <v>86</v>
+      </c>
+      <c r="H46" t="s">
+        <v>228</v>
+      </c>
+      <c r="I46" t="s">
+        <v>26</v>
+      </c>
+      <c r="J46" t="s">
+        <v>26</v>
+      </c>
+      <c r="K46" t="s">
+        <v>26</v>
       </c>
       <c r="L46" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="47" spans="1:12" x14ac:dyDescent="0.35">
+        <v>227</v>
+      </c>
+      <c r="M46" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="47" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A47">
         <v>46</v>
       </c>
       <c r="B47" t="s">
-        <v>103</v>
+        <v>95</v>
       </c>
       <c r="C47">
         <v>1</v>
       </c>
-      <c r="E47" t="s">
-        <v>109</v>
+      <c r="E47">
+        <v>1590</v>
       </c>
       <c r="F47" t="s">
-        <v>94</v>
+        <v>149</v>
+      </c>
+      <c r="G47">
+        <v>1590</v>
+      </c>
+      <c r="H47" t="s">
+        <v>229</v>
+      </c>
+      <c r="I47" t="s">
+        <v>26</v>
+      </c>
+      <c r="J47" t="s">
+        <v>26</v>
+      </c>
+      <c r="K47" t="s">
+        <v>26</v>
       </c>
       <c r="L47" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.35">
+        <v>230</v>
+      </c>
+      <c r="M47" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="48" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A48">
         <v>47</v>
       </c>
       <c r="B48" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
       <c r="C48">
         <v>1</v>
       </c>
       <c r="E48" t="s">
-        <v>110</v>
+        <v>87</v>
       </c>
       <c r="F48" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="G48" t="s">
-        <v>111</v>
+        <v>87</v>
+      </c>
+      <c r="H48" t="s">
+        <v>231</v>
+      </c>
+      <c r="I48" t="s">
+        <v>26</v>
+      </c>
+      <c r="J48" t="s">
+        <v>26</v>
+      </c>
+      <c r="K48" t="s">
+        <v>26</v>
       </c>
       <c r="L48" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
+        <v>26</v>
+      </c>
+      <c r="M48" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="49" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A49">
         <v>48</v>
       </c>
       <c r="B49" t="s">
-        <v>155</v>
+        <v>97</v>
+      </c>
+      <c r="C49">
+        <v>1</v>
       </c>
       <c r="E49" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
+        <v>88</v>
+      </c>
+      <c r="F49" t="s">
+        <v>103</v>
+      </c>
+      <c r="G49" t="s">
+        <v>233</v>
+      </c>
+      <c r="H49" t="s">
+        <v>104</v>
+      </c>
+      <c r="I49" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="J49" t="s">
+        <v>234</v>
+      </c>
+      <c r="K49" t="s">
+        <v>235</v>
+      </c>
+      <c r="L49" t="s">
+        <v>236</v>
+      </c>
+      <c r="M49" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="50" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A50">
         <v>49</v>
       </c>
       <c r="B50" t="s">
-        <v>154</v>
+        <v>148</v>
+      </c>
+      <c r="C50">
+        <v>1</v>
+      </c>
+      <c r="E50" t="s">
+        <v>237</v>
+      </c>
+      <c r="F50" t="s">
+        <v>150</v>
+      </c>
+      <c r="G50" t="s">
+        <v>241</v>
+      </c>
+      <c r="H50" t="s">
+        <v>239</v>
+      </c>
+      <c r="I50" t="s">
+        <v>26</v>
+      </c>
+      <c r="J50" t="s">
+        <v>240</v>
+      </c>
+      <c r="K50" t="s">
+        <v>148</v>
+      </c>
+      <c r="L50" t="s">
+        <v>238</v>
+      </c>
+      <c r="M50" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="51" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A51">
+        <v>50</v>
+      </c>
+      <c r="B51" t="s">
+        <v>147</v>
+      </c>
+      <c r="C51">
+        <v>1</v>
+      </c>
+      <c r="D51">
+        <v>4</v>
+      </c>
+      <c r="E51" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="F51" t="s">
+        <v>149</v>
+      </c>
+      <c r="G51" t="s">
+        <v>243</v>
+      </c>
+      <c r="H51" t="s">
+        <v>244</v>
+      </c>
+      <c r="I51" t="s">
+        <v>26</v>
+      </c>
+      <c r="J51" t="s">
+        <v>26</v>
+      </c>
+      <c r="K51" t="s">
+        <v>26</v>
+      </c>
+      <c r="L51" t="s">
+        <v>245</v>
+      </c>
+      <c r="M51" t="s">
+        <v>80</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <ignoredErrors>
+    <ignoredError sqref="E51" numberStoredAsText="1"/>
+  </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Bom changes - purchase request sent
</commit_message>
<xml_diff>
--- a/hardware/SGI_BOM_V1.1.xlsx
+++ b/hardware/SGI_BOM_V1.1.xlsx
@@ -5,17 +5,17 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ashto\Dev\SeniorDesign_SwanGanz\hardware\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ashton\Dev\SeniorDesign_SwanGanz\hardware\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CCFF16A-C2B2-4BBF-93FD-97B6E7396972}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A0493DF-35AD-4D78-AAC2-9B7A56C9A403}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{4EE8D713-7B25-4092-B83F-8A696BC138B6}"/>
+    <workbookView xWindow="-38520" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{4EE8D713-7B25-4092-B83F-8A696BC138B6}"/>
   </bookViews>
   <sheets>
     <sheet name="Inclusive BOM" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" concurrentCalc="0"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="484" uniqueCount="252">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="513" uniqueCount="261">
   <si>
     <t>Reference</t>
   </si>
@@ -62,9 +62,6 @@
     <t>Footprint</t>
   </si>
   <si>
-    <t>C1, C3, C4, C9, C11, C13, C14, C15, C17, C20, C21, C24, C25, C28, C30, C31, C35, C36, C39</t>
-  </si>
-  <si>
     <t>0.1u</t>
   </si>
   <si>
@@ -89,9 +86,6 @@
     <t>0.01u</t>
   </si>
   <si>
-    <t>C212, C16</t>
-  </si>
-  <si>
     <t>30p</t>
   </si>
   <si>
@@ -170,9 +164,6 @@
     <t>J10</t>
   </si>
   <si>
-    <t>7 POS</t>
-  </si>
-  <si>
     <t>J12</t>
   </si>
   <si>
@@ -404,18 +395,6 @@
     <t>C5, C6, C34, C37</t>
   </si>
   <si>
-    <t>C1206C106J3RACTU</t>
-  </si>
-  <si>
-    <t>KEMET</t>
-  </si>
-  <si>
-    <t>80-C1206C106J3RACTU</t>
-  </si>
-  <si>
-    <t>603-CC0603KRX7R9BB104</t>
-  </si>
-  <si>
     <t>C0G</t>
   </si>
   <si>
@@ -449,9 +428,6 @@
     <t>81-GRM21BR71C475KE1K</t>
   </si>
   <si>
-    <t>5u</t>
-  </si>
-  <si>
     <t>CL31B475KAHNNNE</t>
   </si>
   <si>
@@ -792,6 +768,57 @@
   </si>
   <si>
     <t>71-CRCW0603J-1.8K-E3</t>
+  </si>
+  <si>
+    <t>C1, C3, C4, C9, C11, C13, C14, C15, C17, C20, C21, C24, C25, C28, C30, C31, C33, C35, C36, C39</t>
+  </si>
+  <si>
+    <t>C12, C16</t>
+  </si>
+  <si>
+    <t>81-GCM21B5C1H223FA6L</t>
+  </si>
+  <si>
+    <t>GCM21B5C1H223FA16L</t>
+  </si>
+  <si>
+    <t>C18, C19, C22, C23, C26, C27</t>
+  </si>
+  <si>
+    <t>0.022u</t>
+  </si>
+  <si>
+    <t>Molex</t>
+  </si>
+  <si>
+    <t>MICRO USB</t>
+  </si>
+  <si>
+    <t>MicroUSb</t>
+  </si>
+  <si>
+    <t>538-105164-0001</t>
+  </si>
+  <si>
+    <t>105164-0001</t>
+  </si>
+  <si>
+    <t>1935161</t>
+  </si>
+  <si>
+    <t>603-CC603JRX7R9BB104</t>
+  </si>
+  <si>
+    <t>187-CL31B106MOHNNNE</t>
+  </si>
+  <si>
+    <t>CL31B106MOHNNNE</t>
+  </si>
+  <si>
+    <t>VJ0603Y333KFXAO</t>
+  </si>
+  <si>
+    <t>0.033uF</t>
   </si>
 </sst>
 </file>
@@ -807,7 +834,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -817,6 +844,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -839,7 +872,7 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1174,12 +1207,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2DB84AFE-AA67-459F-9D96-757C0A5835DB}">
-  <dimension ref="A1:M51"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:M53"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="5" max="5" width="27.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="26.42578125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="23.28515625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
@@ -1188,7 +1226,7 @@
         <v>1</v>
       </c>
       <c r="D1" t="s">
-        <v>246</v>
+        <v>238</v>
       </c>
       <c r="E1" t="s">
         <v>2</v>
@@ -1209,1877 +1247,2030 @@
         <v>6</v>
       </c>
       <c r="K1" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="L1" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="M1" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A2">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A2" s="5">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>8</v>
+        <v>244</v>
       </c>
       <c r="C2">
         <v>20</v>
       </c>
+      <c r="D2">
+        <v>100</v>
+      </c>
       <c r="E2" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="F2" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="G2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H2" s="1" t="s">
         <v>9</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>10</v>
       </c>
       <c r="I2" s="4">
         <v>0.05</v>
       </c>
       <c r="J2" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="K2" s="4" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="L2" t="s">
-        <v>125</v>
+        <v>256</v>
       </c>
       <c r="M2" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A3" s="5">
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C3">
         <v>2</v>
       </c>
+      <c r="D3">
+        <v>20</v>
+      </c>
       <c r="E3" t="s">
-        <v>122</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>123</v>
+        <v>258</v>
+      </c>
+      <c r="F3" t="s">
+        <v>115</v>
       </c>
       <c r="G3" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="I3" s="4">
-        <v>0.05</v>
+        <v>0.2</v>
       </c>
       <c r="J3" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="K3" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="L3" t="s">
-        <v>124</v>
+        <v>257</v>
       </c>
       <c r="M3" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A4">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A4" s="5">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="C4">
         <v>4</v>
       </c>
+      <c r="D4">
+        <v>25</v>
+      </c>
       <c r="E4" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="F4" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="G4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="I4" s="4">
         <v>0.1</v>
       </c>
       <c r="J4" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="K4" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="L4" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A5">
+        <v>109</v>
+      </c>
+      <c r="M4" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A5" s="5">
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C5">
         <v>1</v>
       </c>
+      <c r="D5">
+        <v>10</v>
+      </c>
       <c r="E5" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="F5" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="G5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="I5" s="4">
         <v>0.05</v>
       </c>
       <c r="J5" t="s">
+        <v>110</v>
+      </c>
+      <c r="K5" t="s">
+        <v>104</v>
+      </c>
+      <c r="L5" t="s">
         <v>113</v>
       </c>
-      <c r="K5" t="s">
-        <v>107</v>
-      </c>
-      <c r="L5" t="s">
-        <v>116</v>
-      </c>
       <c r="M5" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A6">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A6" s="5">
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C6">
         <v>1</v>
       </c>
+      <c r="D6">
+        <v>10</v>
+      </c>
       <c r="E6" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="F6" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="G6" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="I6" s="4">
         <v>0.1</v>
       </c>
       <c r="J6" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="K6" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="L6" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="M6" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A7">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A7" s="5">
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>17</v>
+        <v>245</v>
       </c>
       <c r="C7">
         <v>2</v>
       </c>
+      <c r="D7">
+        <v>20</v>
+      </c>
       <c r="E7" t="s">
-        <v>127</v>
+        <v>120</v>
       </c>
       <c r="F7" t="s">
-        <v>128</v>
+        <v>121</v>
       </c>
       <c r="G7" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="I7" s="4">
         <v>0.01</v>
       </c>
       <c r="J7" t="s">
-        <v>129</v>
+        <v>122</v>
       </c>
       <c r="K7" t="s">
+        <v>119</v>
+      </c>
+      <c r="L7" t="s">
+        <v>123</v>
+      </c>
+      <c r="M7" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A8" s="5">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>248</v>
+      </c>
+      <c r="C8">
+        <v>6</v>
+      </c>
+      <c r="D8">
+        <v>30</v>
+      </c>
+      <c r="E8" t="s">
+        <v>247</v>
+      </c>
+      <c r="F8" t="s">
+        <v>121</v>
+      </c>
+      <c r="G8" t="s">
+        <v>249</v>
+      </c>
+      <c r="H8" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="L7" t="s">
-        <v>130</v>
-      </c>
-      <c r="M7" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A8">
-        <v>7</v>
-      </c>
-      <c r="B8" t="s">
-        <v>19</v>
-      </c>
-      <c r="C8">
-        <v>1</v>
-      </c>
-      <c r="E8" t="s">
-        <v>131</v>
-      </c>
-      <c r="F8" t="s">
-        <v>128</v>
-      </c>
-      <c r="G8" t="s">
-        <v>20</v>
-      </c>
-      <c r="H8" s="1" t="s">
-        <v>10</v>
-      </c>
       <c r="I8" s="4">
-        <v>0.05</v>
+        <v>0.01</v>
       </c>
       <c r="J8" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="K8" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
       <c r="L8" t="s">
-        <v>132</v>
+        <v>246</v>
       </c>
       <c r="M8" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A9">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A9" s="5">
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="C9">
         <v>1</v>
       </c>
+      <c r="D9">
+        <v>10</v>
+      </c>
       <c r="E9" t="s">
-        <v>134</v>
+        <v>124</v>
+      </c>
+      <c r="F9" t="s">
+        <v>121</v>
       </c>
       <c r="G9" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>133</v>
+        <v>9</v>
       </c>
       <c r="I9" s="4">
-        <v>0.1</v>
+        <v>0.05</v>
       </c>
       <c r="J9" t="s">
-        <v>135</v>
+        <v>105</v>
       </c>
       <c r="K9" t="s">
-        <v>107</v>
+        <v>119</v>
       </c>
       <c r="L9" t="s">
-        <v>136</v>
+        <v>125</v>
       </c>
       <c r="M9" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A10">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A10" s="5">
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C10">
         <v>1</v>
       </c>
+      <c r="D10">
+        <v>10</v>
+      </c>
       <c r="E10" t="s">
-        <v>138</v>
+        <v>127</v>
       </c>
       <c r="F10" t="s">
-        <v>128</v>
+        <v>121</v>
       </c>
       <c r="G10" t="s">
-        <v>137</v>
+        <v>20</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>24</v>
+        <v>126</v>
       </c>
       <c r="I10" s="4">
         <v>0.1</v>
       </c>
       <c r="J10" t="s">
-        <v>113</v>
+        <v>128</v>
       </c>
       <c r="K10" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="L10" t="s">
-        <v>139</v>
+        <v>129</v>
       </c>
       <c r="M10" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A11">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A11" s="5">
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="C11">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="D11">
+        <v>10</v>
       </c>
       <c r="E11" t="s">
-        <v>27</v>
+        <v>130</v>
       </c>
       <c r="F11" t="s">
-        <v>27</v>
+        <v>121</v>
       </c>
       <c r="G11" t="s">
-        <v>26</v>
-      </c>
-      <c r="H11" t="s">
-        <v>25</v>
-      </c>
-      <c r="I11" t="s">
-        <v>26</v>
+        <v>20</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="I11" s="4">
+        <v>0.1</v>
       </c>
       <c r="J11" t="s">
-        <v>26</v>
+        <v>110</v>
       </c>
       <c r="K11" t="s">
-        <v>26</v>
+        <v>104</v>
       </c>
       <c r="L11" t="s">
-        <v>26</v>
+        <v>131</v>
       </c>
       <c r="M11" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.35">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C12">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="D12" t="s">
+        <v>24</v>
       </c>
       <c r="E12" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="F12" t="s">
-        <v>140</v>
+        <v>25</v>
       </c>
       <c r="G12" t="s">
-        <v>141</v>
-      </c>
-      <c r="H12" s="1" t="s">
-        <v>10</v>
+        <v>24</v>
+      </c>
+      <c r="H12" t="s">
+        <v>23</v>
       </c>
       <c r="I12" t="s">
+        <v>24</v>
+      </c>
+      <c r="J12" t="s">
+        <v>24</v>
+      </c>
+      <c r="K12" t="s">
+        <v>24</v>
+      </c>
+      <c r="L12" t="s">
+        <v>24</v>
+      </c>
+      <c r="M12" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A13" s="5">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
         <v>26</v>
-      </c>
-      <c r="J12" t="s">
-        <v>142</v>
-      </c>
-      <c r="K12" t="s">
-        <v>143</v>
-      </c>
-      <c r="L12" t="s">
-        <v>144</v>
-      </c>
-      <c r="M12" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A13">
-        <v>12</v>
-      </c>
-      <c r="B13" t="s">
-        <v>32</v>
       </c>
       <c r="C13">
         <v>1</v>
       </c>
+      <c r="D13">
+        <v>10</v>
+      </c>
       <c r="E13" t="s">
+        <v>27</v>
+      </c>
+      <c r="F13" t="s">
+        <v>132</v>
+      </c>
+      <c r="G13" t="s">
+        <v>133</v>
+      </c>
+      <c r="H13" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="I13" t="s">
+        <v>24</v>
+      </c>
+      <c r="J13" t="s">
+        <v>134</v>
+      </c>
+      <c r="K13" t="s">
+        <v>135</v>
+      </c>
+      <c r="L13" t="s">
+        <v>136</v>
+      </c>
+      <c r="M13" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A14" s="5">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
         <v>30</v>
-      </c>
-      <c r="F13" t="s">
-        <v>140</v>
-      </c>
-      <c r="G13" t="s">
-        <v>146</v>
-      </c>
-      <c r="H13" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="I13" t="s">
-        <v>26</v>
-      </c>
-      <c r="J13" t="s">
-        <v>142</v>
-      </c>
-      <c r="K13" t="s">
-        <v>143</v>
-      </c>
-      <c r="L13" t="s">
-        <v>145</v>
-      </c>
-      <c r="M13" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A14">
-        <v>13</v>
-      </c>
-      <c r="B14" t="s">
-        <v>33</v>
       </c>
       <c r="C14">
         <v>1</v>
       </c>
+      <c r="D14">
+        <v>10</v>
+      </c>
       <c r="E14" t="s">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="F14" t="s">
-        <v>27</v>
+        <v>132</v>
       </c>
       <c r="G14" t="s">
-        <v>35</v>
-      </c>
-      <c r="H14" t="s">
-        <v>34</v>
+        <v>138</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>9</v>
       </c>
       <c r="I14" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="J14" t="s">
-        <v>26</v>
+        <v>134</v>
       </c>
       <c r="K14" t="s">
-        <v>26</v>
+        <v>135</v>
       </c>
       <c r="L14" t="s">
-        <v>26</v>
+        <v>137</v>
       </c>
       <c r="M14" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.35">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>14</v>
       </c>
       <c r="B15" t="s">
+        <v>31</v>
+      </c>
+      <c r="C15">
+        <v>1</v>
+      </c>
+      <c r="D15" t="s">
+        <v>24</v>
+      </c>
+      <c r="E15" t="s">
         <v>36</v>
       </c>
-      <c r="C15">
-        <v>2</v>
-      </c>
-      <c r="E15" t="s">
-        <v>26</v>
-      </c>
       <c r="F15" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G15" t="s">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="H15" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="I15" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="J15" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="K15" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="L15" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="M15" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.35">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="C16">
         <v>2</v>
       </c>
+      <c r="D16" t="s">
+        <v>24</v>
+      </c>
       <c r="E16" t="s">
-        <v>39</v>
+        <v>24</v>
       </c>
       <c r="F16" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="G16" t="s">
-        <v>40</v>
+        <v>24</v>
       </c>
       <c r="H16" t="s">
-        <v>34</v>
+        <v>24</v>
       </c>
       <c r="I16" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="J16" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="K16" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="L16" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="M16" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.35">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="C17">
         <v>2</v>
       </c>
+      <c r="D17" t="s">
+        <v>24</v>
+      </c>
       <c r="E17" t="s">
+        <v>37</v>
+      </c>
+      <c r="F17" t="s">
+        <v>25</v>
+      </c>
+      <c r="G17" t="s">
         <v>38</v>
       </c>
-      <c r="F17" t="s">
-        <v>42</v>
-      </c>
-      <c r="G17" t="s">
-        <v>40</v>
-      </c>
       <c r="H17" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="I17" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="J17" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="K17" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="L17" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="M17" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.35">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="C18">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="D18" t="s">
+        <v>24</v>
       </c>
       <c r="E18" t="s">
+        <v>36</v>
+      </c>
+      <c r="F18" t="s">
+        <v>40</v>
+      </c>
+      <c r="G18" t="s">
         <v>38</v>
       </c>
-      <c r="F18" t="s">
-        <v>27</v>
-      </c>
-      <c r="G18" t="s">
-        <v>44</v>
-      </c>
       <c r="H18" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="I18" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="J18" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="K18" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="L18" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="M18" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A19">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A19" s="5">
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="C19">
         <v>1</v>
       </c>
+      <c r="D19">
+        <v>10</v>
+      </c>
       <c r="E19" t="s">
-        <v>38</v>
+        <v>254</v>
       </c>
       <c r="F19" t="s">
-        <v>27</v>
+        <v>250</v>
       </c>
       <c r="G19" t="s">
-        <v>46</v>
+        <v>251</v>
       </c>
       <c r="H19" t="s">
-        <v>34</v>
+        <v>252</v>
       </c>
       <c r="I19" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="J19" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="K19" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="L19" t="s">
-        <v>26</v>
+        <v>253</v>
       </c>
       <c r="M19" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.35">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="C20">
         <v>1</v>
       </c>
-      <c r="E20">
-        <v>1935161</v>
+      <c r="D20" t="s">
+        <v>24</v>
+      </c>
+      <c r="E20" t="s">
+        <v>36</v>
       </c>
       <c r="F20" t="s">
-        <v>151</v>
+        <v>25</v>
       </c>
       <c r="G20" t="s">
-        <v>152</v>
+        <v>43</v>
       </c>
       <c r="H20" t="s">
-        <v>153</v>
+        <v>32</v>
       </c>
       <c r="I20" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="J20" t="s">
-        <v>154</v>
+        <v>24</v>
       </c>
       <c r="K20" t="s">
-        <v>48</v>
+        <v>24</v>
       </c>
       <c r="L20" t="s">
-        <v>155</v>
+        <v>24</v>
       </c>
       <c r="M20" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A21">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A21" s="5">
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>158</v>
+        <v>44</v>
       </c>
       <c r="C21">
         <v>1</v>
       </c>
-      <c r="E21" t="s">
+      <c r="D21">
+        <v>8</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>255</v>
+      </c>
+      <c r="F21" t="s">
+        <v>143</v>
+      </c>
+      <c r="G21" t="s">
+        <v>144</v>
+      </c>
+      <c r="H21" t="s">
+        <v>145</v>
+      </c>
+      <c r="I21" t="s">
+        <v>24</v>
+      </c>
+      <c r="J21" t="s">
+        <v>146</v>
+      </c>
+      <c r="K21" t="s">
+        <v>45</v>
+      </c>
+      <c r="L21" t="s">
+        <v>147</v>
+      </c>
+      <c r="M21" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A22" s="5">
+        <v>21</v>
+      </c>
+      <c r="B22" t="s">
+        <v>150</v>
+      </c>
+      <c r="C22">
+        <v>1</v>
+      </c>
+      <c r="D22">
+        <v>10</v>
+      </c>
+      <c r="E22" t="s">
+        <v>48</v>
+      </c>
+      <c r="F22" t="s">
+        <v>151</v>
+      </c>
+      <c r="G22" t="s">
+        <v>152</v>
+      </c>
+      <c r="H22" t="s">
+        <v>96</v>
+      </c>
+      <c r="I22" t="s">
+        <v>24</v>
+      </c>
+      <c r="J22" t="s">
+        <v>149</v>
+      </c>
+      <c r="K22" t="s">
+        <v>49</v>
+      </c>
+      <c r="L22" t="s">
+        <v>148</v>
+      </c>
+      <c r="M22" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A23" s="5">
+        <v>22</v>
+      </c>
+      <c r="B23" t="s">
+        <v>50</v>
+      </c>
+      <c r="C23">
+        <v>2</v>
+      </c>
+      <c r="D23">
+        <v>20</v>
+      </c>
+      <c r="E23" t="s">
+        <v>153</v>
+      </c>
+      <c r="F23" t="s">
+        <v>112</v>
+      </c>
+      <c r="G23" t="s">
         <v>51</v>
       </c>
-      <c r="F21" t="s">
-        <v>159</v>
-      </c>
-      <c r="G21" t="s">
-        <v>160</v>
-      </c>
-      <c r="H21" t="s">
-        <v>99</v>
-      </c>
-      <c r="I21" t="s">
-        <v>26</v>
-      </c>
-      <c r="J21" t="s">
-        <v>157</v>
-      </c>
-      <c r="K21" t="s">
-        <v>52</v>
-      </c>
-      <c r="L21" t="s">
-        <v>156</v>
-      </c>
-      <c r="M21" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A22">
-        <v>21</v>
-      </c>
-      <c r="B22" t="s">
-        <v>53</v>
-      </c>
-      <c r="C22">
-        <v>2</v>
-      </c>
-      <c r="E22" t="s">
-        <v>161</v>
-      </c>
-      <c r="F22" t="s">
-        <v>115</v>
-      </c>
-      <c r="G22" t="s">
-        <v>54</v>
-      </c>
-      <c r="H22" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="I22" s="3">
-        <v>5.0000000000000001E-3</v>
-      </c>
-      <c r="J22" t="s">
-        <v>162</v>
-      </c>
-      <c r="K22" t="s">
-        <v>163</v>
-      </c>
-      <c r="L22" t="s">
-        <v>164</v>
-      </c>
-      <c r="M22" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A23">
-        <v>22</v>
-      </c>
-      <c r="B23" t="s">
-        <v>55</v>
-      </c>
-      <c r="C23">
-        <v>13</v>
-      </c>
-      <c r="E23" t="s">
-        <v>165</v>
-      </c>
-      <c r="F23" t="s">
-        <v>115</v>
-      </c>
-      <c r="G23" t="s">
-        <v>63</v>
-      </c>
       <c r="H23" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="I23" s="3">
         <v>5.0000000000000001E-3</v>
       </c>
       <c r="J23" t="s">
-        <v>162</v>
+        <v>154</v>
       </c>
       <c r="K23" t="s">
-        <v>163</v>
+        <v>155</v>
       </c>
       <c r="L23" t="s">
-        <v>166</v>
+        <v>156</v>
       </c>
       <c r="M23" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A24">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A24" s="5">
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>249</v>
+        <v>52</v>
       </c>
       <c r="C24">
-        <v>3</v>
+        <v>13</v>
+      </c>
+      <c r="D24">
+        <v>100</v>
       </c>
       <c r="E24" t="s">
-        <v>167</v>
+        <v>157</v>
       </c>
       <c r="F24" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="G24" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="H24" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="I24" s="3">
         <v>5.0000000000000001E-3</v>
       </c>
       <c r="J24" t="s">
+        <v>154</v>
+      </c>
+      <c r="K24" t="s">
+        <v>155</v>
+      </c>
+      <c r="L24" t="s">
+        <v>158</v>
+      </c>
+      <c r="M24" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A25" s="5">
+        <v>24</v>
+      </c>
+      <c r="B25" t="s">
+        <v>241</v>
+      </c>
+      <c r="C25">
+        <v>3</v>
+      </c>
+      <c r="D25">
+        <v>25</v>
+      </c>
+      <c r="E25" t="s">
+        <v>159</v>
+      </c>
+      <c r="F25" t="s">
+        <v>112</v>
+      </c>
+      <c r="G25" t="s">
+        <v>61</v>
+      </c>
+      <c r="H25" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="I25" s="3">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="J25" t="s">
+        <v>154</v>
+      </c>
+      <c r="K25" t="s">
+        <v>155</v>
+      </c>
+      <c r="L25" t="s">
+        <v>160</v>
+      </c>
+      <c r="M25" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A26" s="5">
+        <v>25</v>
+      </c>
+      <c r="B26" t="s">
+        <v>177</v>
+      </c>
+      <c r="C26">
+        <v>1</v>
+      </c>
+      <c r="D26">
+        <v>10</v>
+      </c>
+      <c r="E26" t="s">
+        <v>181</v>
+      </c>
+      <c r="F26" t="s">
+        <v>167</v>
+      </c>
+      <c r="G26" t="s">
+        <v>62</v>
+      </c>
+      <c r="H26" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="I26" s="3">
+        <v>1E-3</v>
+      </c>
+      <c r="J26" t="s">
+        <v>172</v>
+      </c>
+      <c r="K26" t="s">
+        <v>155</v>
+      </c>
+      <c r="L26" t="s">
+        <v>183</v>
+      </c>
+      <c r="M26" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A27" s="5">
+        <v>26</v>
+      </c>
+      <c r="B27" t="s">
+        <v>182</v>
+      </c>
+      <c r="C27">
+        <v>15</v>
+      </c>
+      <c r="D27">
+        <v>50</v>
+      </c>
+      <c r="E27" t="s">
         <v>162</v>
       </c>
-      <c r="K24" t="s">
+      <c r="F27" t="s">
+        <v>112</v>
+      </c>
+      <c r="G27" t="s">
+        <v>62</v>
+      </c>
+      <c r="H27" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="I27" s="3">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="J27" t="s">
+        <v>154</v>
+      </c>
+      <c r="K27" t="s">
+        <v>155</v>
+      </c>
+      <c r="L27" t="s">
+        <v>161</v>
+      </c>
+      <c r="M27" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A28" s="5">
+        <v>27</v>
+      </c>
+      <c r="B28" t="s">
+        <v>53</v>
+      </c>
+      <c r="C28">
+        <v>5</v>
+      </c>
+      <c r="D28">
+        <v>50</v>
+      </c>
+      <c r="E28" t="s">
         <v>163</v>
       </c>
-      <c r="L24" t="s">
-        <v>168</v>
-      </c>
-      <c r="M24" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A25">
-        <v>24</v>
-      </c>
-      <c r="B25" t="s">
-        <v>185</v>
-      </c>
-      <c r="C25">
-        <v>1</v>
-      </c>
-      <c r="E25" t="s">
-        <v>189</v>
-      </c>
-      <c r="F25" t="s">
-        <v>175</v>
-      </c>
-      <c r="G25" t="s">
-        <v>65</v>
-      </c>
-      <c r="H25" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="I25" s="3">
-        <v>1E-3</v>
-      </c>
-      <c r="J25" t="s">
-        <v>180</v>
-      </c>
-      <c r="K25" t="s">
-        <v>163</v>
-      </c>
-      <c r="L25" t="s">
-        <v>191</v>
-      </c>
-      <c r="M25" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A26">
-        <v>25</v>
-      </c>
-      <c r="B26" t="s">
-        <v>190</v>
-      </c>
-      <c r="C26">
-        <v>15</v>
-      </c>
-      <c r="E26" t="s">
-        <v>170</v>
-      </c>
-      <c r="F26" t="s">
-        <v>115</v>
-      </c>
-      <c r="G26" t="s">
-        <v>65</v>
-      </c>
-      <c r="H26" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="I26" s="3">
-        <v>5.0000000000000001E-3</v>
-      </c>
-      <c r="J26" t="s">
-        <v>162</v>
-      </c>
-      <c r="K26" t="s">
-        <v>163</v>
-      </c>
-      <c r="L26" t="s">
-        <v>169</v>
-      </c>
-      <c r="M26" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A27">
-        <v>26</v>
-      </c>
-      <c r="B27" t="s">
-        <v>56</v>
-      </c>
-      <c r="C27">
-        <v>5</v>
-      </c>
-      <c r="E27" t="s">
-        <v>171</v>
-      </c>
-      <c r="F27" t="s">
-        <v>159</v>
-      </c>
-      <c r="G27" t="s">
-        <v>66</v>
-      </c>
-      <c r="H27" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="I27" s="4">
+      <c r="F28" t="s">
+        <v>151</v>
+      </c>
+      <c r="G28" t="s">
+        <v>63</v>
+      </c>
+      <c r="H28" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="I28" s="4">
         <v>0.01</v>
       </c>
-      <c r="J27" t="s">
-        <v>172</v>
-      </c>
-      <c r="K27" t="s">
-        <v>163</v>
-      </c>
-      <c r="L27" t="s">
-        <v>173</v>
-      </c>
-      <c r="M27" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A28">
-        <v>27</v>
-      </c>
-      <c r="B28" t="s">
-        <v>57</v>
-      </c>
-      <c r="C28">
+      <c r="J28" t="s">
+        <v>164</v>
+      </c>
+      <c r="K28" t="s">
+        <v>155</v>
+      </c>
+      <c r="L28" t="s">
+        <v>165</v>
+      </c>
+      <c r="M28" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A29" s="5">
+        <v>28</v>
+      </c>
+      <c r="B29" t="s">
+        <v>54</v>
+      </c>
+      <c r="C29">
         <v>2</v>
       </c>
-      <c r="E28" t="s">
-        <v>174</v>
-      </c>
-      <c r="F28" t="s">
-        <v>175</v>
-      </c>
-      <c r="G28" t="s">
-        <v>67</v>
-      </c>
-      <c r="H28" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="I28" s="3">
-        <v>5.0000000000000001E-3</v>
-      </c>
-      <c r="J28" t="s">
-        <v>162</v>
-      </c>
-      <c r="K28" t="s">
-        <v>163</v>
-      </c>
-      <c r="L28" t="s">
-        <v>176</v>
-      </c>
-      <c r="M28" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A29">
-        <v>28</v>
-      </c>
-      <c r="B29" t="s">
-        <v>58</v>
-      </c>
-      <c r="C29">
-        <v>1</v>
+      <c r="D29">
+        <v>20</v>
       </c>
       <c r="E29" t="s">
-        <v>177</v>
+        <v>166</v>
       </c>
       <c r="F29" t="s">
-        <v>115</v>
+        <v>167</v>
       </c>
       <c r="G29" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="H29" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="I29" s="3">
         <v>5.0000000000000001E-3</v>
       </c>
       <c r="J29" t="s">
-        <v>162</v>
+        <v>154</v>
       </c>
       <c r="K29" t="s">
-        <v>163</v>
+        <v>155</v>
       </c>
       <c r="L29" t="s">
-        <v>178</v>
+        <v>168</v>
       </c>
       <c r="M29" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A30">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A30" s="5">
         <v>29</v>
       </c>
       <c r="B30" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="C30">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="D30">
+        <v>10</v>
       </c>
       <c r="E30" t="s">
-        <v>179</v>
+        <v>169</v>
       </c>
       <c r="F30" t="s">
-        <v>175</v>
+        <v>112</v>
       </c>
       <c r="G30" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="H30" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="I30" s="3">
         <v>5.0000000000000001E-3</v>
       </c>
       <c r="J30" t="s">
-        <v>180</v>
+        <v>154</v>
       </c>
       <c r="K30" t="s">
-        <v>163</v>
+        <v>155</v>
       </c>
       <c r="L30" t="s">
-        <v>181</v>
+        <v>170</v>
       </c>
       <c r="M30" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A31">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A31" s="5">
         <v>30</v>
       </c>
       <c r="B31" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="C31">
         <v>2</v>
       </c>
+      <c r="D31">
+        <v>20</v>
+      </c>
       <c r="E31" t="s">
-        <v>184</v>
+        <v>171</v>
       </c>
       <c r="F31" t="s">
-        <v>175</v>
+        <v>167</v>
       </c>
       <c r="G31" t="s">
-        <v>183</v>
+        <v>66</v>
       </c>
       <c r="H31" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="I31" s="3">
         <v>5.0000000000000001E-3</v>
       </c>
       <c r="J31" t="s">
-        <v>180</v>
+        <v>172</v>
       </c>
       <c r="K31" t="s">
-        <v>163</v>
+        <v>155</v>
       </c>
       <c r="L31" t="s">
-        <v>182</v>
+        <v>173</v>
       </c>
       <c r="M31" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A32">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A32" s="5">
         <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="C32">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="D32">
+        <v>20</v>
       </c>
       <c r="E32" t="s">
-        <v>188</v>
+        <v>176</v>
       </c>
       <c r="F32" t="s">
-        <v>187</v>
+        <v>167</v>
       </c>
       <c r="G32" t="s">
-        <v>62</v>
+        <v>175</v>
       </c>
       <c r="H32" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="I32" s="4">
-        <v>0.05</v>
+        <v>9</v>
+      </c>
+      <c r="I32" s="3">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="J32" t="s">
-        <v>162</v>
+        <v>172</v>
       </c>
       <c r="K32" t="s">
-        <v>163</v>
+        <v>155</v>
       </c>
       <c r="L32" t="s">
-        <v>186</v>
+        <v>174</v>
       </c>
       <c r="M32" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A33">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A33" s="5">
         <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>248</v>
+        <v>58</v>
       </c>
       <c r="C33">
         <v>1</v>
       </c>
+      <c r="D33">
+        <v>10</v>
+      </c>
       <c r="E33" t="s">
-        <v>250</v>
+        <v>180</v>
       </c>
       <c r="F33" t="s">
-        <v>159</v>
-      </c>
-      <c r="G33" s="2" t="s">
-        <v>247</v>
+        <v>179</v>
+      </c>
+      <c r="G33" t="s">
+        <v>59</v>
       </c>
       <c r="H33" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="I33" s="4">
         <v>0.05</v>
       </c>
       <c r="J33" t="s">
-        <v>172</v>
+        <v>154</v>
       </c>
       <c r="K33" t="s">
-        <v>163</v>
+        <v>155</v>
       </c>
       <c r="L33" t="s">
-        <v>251</v>
+        <v>178</v>
       </c>
       <c r="M33" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A34">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A34" s="5">
         <v>33</v>
       </c>
       <c r="B34" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="C34">
         <v>1</v>
       </c>
+      <c r="D34">
+        <v>10</v>
+      </c>
       <c r="E34" t="s">
-        <v>197</v>
+        <v>189</v>
       </c>
       <c r="F34" t="s">
-        <v>196</v>
+        <v>188</v>
       </c>
       <c r="G34" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="H34" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="I34" t="s">
+        <v>187</v>
+      </c>
+      <c r="J34" t="s">
+        <v>185</v>
+      </c>
+      <c r="K34" t="s">
+        <v>155</v>
+      </c>
+      <c r="L34" t="s">
+        <v>184</v>
+      </c>
+      <c r="M34" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="35" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A35" s="5">
+        <v>34</v>
+      </c>
+      <c r="B35" t="s">
+        <v>240</v>
+      </c>
+      <c r="C35">
+        <v>1</v>
+      </c>
+      <c r="D35">
         <v>10</v>
       </c>
-      <c r="I34" t="s">
-        <v>195</v>
-      </c>
-      <c r="J34" t="s">
-        <v>193</v>
-      </c>
-      <c r="K34" t="s">
-        <v>163</v>
-      </c>
-      <c r="L34" t="s">
-        <v>192</v>
-      </c>
-      <c r="M34" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A35">
-        <v>34</v>
-      </c>
-      <c r="B35" t="s">
-        <v>71</v>
-      </c>
-      <c r="C35">
+      <c r="E35" t="s">
+        <v>242</v>
+      </c>
+      <c r="F35" t="s">
+        <v>151</v>
+      </c>
+      <c r="G35" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="H35" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="I35" s="4">
+        <v>0.05</v>
+      </c>
+      <c r="J35" t="s">
+        <v>164</v>
+      </c>
+      <c r="K35" t="s">
+        <v>155</v>
+      </c>
+      <c r="L35" t="s">
+        <v>243</v>
+      </c>
+      <c r="M35" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="36" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A36" s="5">
+        <v>35</v>
+      </c>
+      <c r="B36" t="s">
+        <v>68</v>
+      </c>
+      <c r="C36">
         <v>2</v>
       </c>
-      <c r="E35" t="s">
-        <v>198</v>
-      </c>
-      <c r="F35" t="s">
-        <v>199</v>
-      </c>
-      <c r="G35" t="s">
-        <v>72</v>
-      </c>
-      <c r="H35" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="I35" s="4">
-        <v>0.01</v>
-      </c>
-      <c r="J35" t="s">
-        <v>162</v>
-      </c>
-      <c r="K35" t="s">
-        <v>163</v>
-      </c>
-      <c r="L35" t="s">
-        <v>200</v>
-      </c>
-      <c r="M35" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A36">
-        <v>35</v>
-      </c>
-      <c r="B36" t="s">
-        <v>74</v>
-      </c>
-      <c r="C36">
-        <v>1</v>
+      <c r="D36">
+        <v>20</v>
       </c>
       <c r="E36" t="s">
-        <v>201</v>
+        <v>190</v>
       </c>
       <c r="F36" t="s">
-        <v>202</v>
+        <v>191</v>
       </c>
       <c r="G36" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="H36" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="I36" s="4">
         <v>0.01</v>
       </c>
       <c r="J36" t="s">
-        <v>162</v>
+        <v>154</v>
       </c>
       <c r="K36" t="s">
-        <v>163</v>
+        <v>155</v>
       </c>
       <c r="L36" t="s">
-        <v>203</v>
+        <v>192</v>
       </c>
       <c r="M36" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="37" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A37">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="37" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A37" s="5">
         <v>36</v>
       </c>
       <c r="B37" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="C37">
         <v>1</v>
       </c>
+      <c r="D37">
+        <v>10</v>
+      </c>
       <c r="E37" t="s">
-        <v>206</v>
+        <v>193</v>
       </c>
       <c r="F37" t="s">
-        <v>205</v>
+        <v>194</v>
       </c>
       <c r="G37" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="H37" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="I37" s="4">
         <v>0.01</v>
       </c>
       <c r="J37" t="s">
-        <v>162</v>
+        <v>154</v>
       </c>
       <c r="K37" t="s">
-        <v>163</v>
+        <v>155</v>
       </c>
       <c r="L37" t="s">
-        <v>204</v>
+        <v>195</v>
       </c>
       <c r="M37" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="38" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A38">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="38" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A38" s="5">
         <v>37</v>
       </c>
       <c r="B38" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="C38">
         <v>1</v>
       </c>
+      <c r="D38">
+        <v>10</v>
+      </c>
       <c r="E38" t="s">
-        <v>77</v>
+        <v>198</v>
       </c>
       <c r="F38" t="s">
-        <v>207</v>
+        <v>197</v>
       </c>
       <c r="G38" t="s">
-        <v>77</v>
-      </c>
-      <c r="H38" t="s">
-        <v>26</v>
-      </c>
-      <c r="I38" t="s">
-        <v>26</v>
+        <v>73</v>
+      </c>
+      <c r="H38" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="I38" s="4">
+        <v>0.01</v>
       </c>
       <c r="J38" t="s">
-        <v>194</v>
+        <v>154</v>
       </c>
       <c r="K38" t="s">
-        <v>208</v>
+        <v>155</v>
       </c>
       <c r="L38" t="s">
-        <v>209</v>
+        <v>196</v>
       </c>
       <c r="M38" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="39" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A39">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="39" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A39" s="5">
         <v>38</v>
       </c>
       <c r="B39" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="C39">
-        <v>5</v>
+        <v>1</v>
+      </c>
+      <c r="D39">
+        <v>10</v>
       </c>
       <c r="E39" t="s">
-        <v>27</v>
+        <v>74</v>
       </c>
       <c r="F39" t="s">
-        <v>27</v>
+        <v>199</v>
       </c>
       <c r="G39" t="s">
-        <v>26</v>
+        <v>74</v>
       </c>
       <c r="H39" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="I39" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="J39" t="s">
-        <v>26</v>
+        <v>186</v>
       </c>
       <c r="K39" t="s">
-        <v>26</v>
+        <v>200</v>
       </c>
       <c r="L39" t="s">
-        <v>26</v>
+        <v>201</v>
       </c>
       <c r="M39" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="40" spans="1:13" x14ac:dyDescent="0.35">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="40" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>39</v>
       </c>
       <c r="B40" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="C40">
-        <v>1</v>
+        <v>5</v>
+      </c>
+      <c r="D40" t="s">
+        <v>24</v>
       </c>
       <c r="E40" t="s">
-        <v>214</v>
+        <v>25</v>
       </c>
       <c r="F40" t="s">
-        <v>101</v>
+        <v>25</v>
       </c>
       <c r="G40" t="s">
-        <v>215</v>
+        <v>24</v>
       </c>
       <c r="H40" t="s">
-        <v>210</v>
+        <v>24</v>
       </c>
       <c r="I40" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="J40" t="s">
-        <v>211</v>
+        <v>24</v>
       </c>
       <c r="K40" t="s">
-        <v>213</v>
+        <v>24</v>
       </c>
       <c r="L40" t="s">
-        <v>212</v>
+        <v>24</v>
       </c>
       <c r="M40" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="41" spans="1:13" x14ac:dyDescent="0.35">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="41" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>40</v>
       </c>
       <c r="B41" t="s">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="C41">
         <v>1</v>
       </c>
+      <c r="D41" t="s">
+        <v>24</v>
+      </c>
       <c r="E41" t="s">
-        <v>82</v>
+        <v>206</v>
       </c>
       <c r="F41" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="G41" t="s">
-        <v>82</v>
+        <v>207</v>
       </c>
       <c r="H41" t="s">
-        <v>216</v>
+        <v>202</v>
       </c>
       <c r="I41" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="J41" t="s">
-        <v>26</v>
+        <v>203</v>
       </c>
       <c r="K41" t="s">
-        <v>26</v>
+        <v>205</v>
       </c>
       <c r="L41" t="s">
-        <v>217</v>
+        <v>204</v>
       </c>
       <c r="M41" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="42" spans="1:13" x14ac:dyDescent="0.35">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="42" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>41</v>
       </c>
       <c r="B42" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="C42">
-        <v>5</v>
+        <v>1</v>
+      </c>
+      <c r="D42" t="s">
+        <v>24</v>
       </c>
       <c r="E42" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="F42" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="G42" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="H42" t="s">
-        <v>222</v>
+        <v>208</v>
       </c>
       <c r="I42" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="J42" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="K42" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="L42" t="s">
-        <v>26</v>
+        <v>209</v>
       </c>
       <c r="M42" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="43" spans="1:13" x14ac:dyDescent="0.35">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="43" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>42</v>
       </c>
       <c r="B43" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="C43">
+        <v>5</v>
+      </c>
+      <c r="D43" t="s">
+        <v>24</v>
+      </c>
+      <c r="E43" t="s">
+        <v>80</v>
+      </c>
+      <c r="F43" t="s">
+        <v>98</v>
+      </c>
+      <c r="G43" t="s">
+        <v>80</v>
+      </c>
+      <c r="H43" t="s">
+        <v>214</v>
+      </c>
+      <c r="I43" t="s">
+        <v>24</v>
+      </c>
+      <c r="J43" t="s">
+        <v>24</v>
+      </c>
+      <c r="K43" t="s">
+        <v>24</v>
+      </c>
+      <c r="L43" t="s">
+        <v>24</v>
+      </c>
+      <c r="M43" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="44" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A44" s="5">
+        <v>43</v>
+      </c>
+      <c r="B44" t="s">
+        <v>88</v>
+      </c>
+      <c r="C44">
         <v>1</v>
       </c>
-      <c r="E43" t="s">
-        <v>218</v>
-      </c>
-      <c r="F43" t="s">
-        <v>101</v>
-      </c>
-      <c r="G43" t="s">
-        <v>26</v>
-      </c>
-      <c r="H43" t="s">
-        <v>219</v>
-      </c>
-      <c r="I43" t="s">
-        <v>26</v>
-      </c>
-      <c r="J43" t="s">
-        <v>26</v>
-      </c>
-      <c r="K43" t="s">
-        <v>26</v>
-      </c>
-      <c r="L43" t="s">
-        <v>220</v>
-      </c>
-      <c r="M43" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="44" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A44">
-        <v>43</v>
-      </c>
-      <c r="B44" t="s">
-        <v>92</v>
-      </c>
-      <c r="C44">
-        <v>3</v>
+      <c r="D44">
+        <v>15</v>
       </c>
       <c r="E44" t="s">
-        <v>84</v>
+        <v>210</v>
       </c>
       <c r="F44" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="G44" t="s">
-        <v>84</v>
+        <v>24</v>
       </c>
       <c r="H44" t="s">
-        <v>222</v>
+        <v>211</v>
       </c>
       <c r="I44" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="J44" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="K44" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="L44" t="s">
-        <v>221</v>
+        <v>212</v>
       </c>
       <c r="M44" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="45" spans="1:13" x14ac:dyDescent="0.35">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="45" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>44</v>
       </c>
       <c r="B45" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="C45">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="D45" t="s">
+        <v>24</v>
       </c>
       <c r="E45" t="s">
-        <v>224</v>
+        <v>81</v>
       </c>
       <c r="F45" t="s">
-        <v>225</v>
+        <v>98</v>
       </c>
       <c r="G45" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="H45" t="s">
-        <v>226</v>
+        <v>214</v>
       </c>
       <c r="I45" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="J45" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="K45" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="L45" t="s">
-        <v>223</v>
+        <v>213</v>
       </c>
       <c r="M45" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="46" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A46">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="46" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A46" s="5">
         <v>45</v>
       </c>
       <c r="B46" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="C46">
         <v>1</v>
       </c>
+      <c r="D46">
+        <v>15</v>
+      </c>
       <c r="E46" t="s">
-        <v>86</v>
+        <v>216</v>
       </c>
       <c r="F46" t="s">
-        <v>101</v>
+        <v>217</v>
       </c>
       <c r="G46" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="H46" t="s">
-        <v>228</v>
+        <v>218</v>
       </c>
       <c r="I46" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="J46" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="K46" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="L46" t="s">
-        <v>227</v>
+        <v>215</v>
       </c>
       <c r="M46" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="47" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A47">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="47" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A47" s="5">
         <v>46</v>
       </c>
       <c r="B47" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="C47">
         <v>1</v>
       </c>
-      <c r="E47">
-        <v>1590</v>
+      <c r="D47">
+        <v>10</v>
+      </c>
+      <c r="E47" t="s">
+        <v>83</v>
       </c>
       <c r="F47" t="s">
-        <v>149</v>
-      </c>
-      <c r="G47">
-        <v>1590</v>
+        <v>98</v>
+      </c>
+      <c r="G47" t="s">
+        <v>83</v>
       </c>
       <c r="H47" t="s">
-        <v>229</v>
+        <v>220</v>
       </c>
       <c r="I47" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="J47" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="K47" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="L47" t="s">
-        <v>230</v>
+        <v>219</v>
       </c>
       <c r="M47" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="48" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A48">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="48" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A48" s="5">
         <v>47</v>
       </c>
       <c r="B48" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="C48">
         <v>1</v>
       </c>
-      <c r="E48" t="s">
-        <v>87</v>
+      <c r="D48">
+        <v>3</v>
+      </c>
+      <c r="E48">
+        <v>1590</v>
       </c>
       <c r="F48" t="s">
-        <v>102</v>
-      </c>
-      <c r="G48" t="s">
-        <v>87</v>
+        <v>141</v>
+      </c>
+      <c r="G48">
+        <v>1590</v>
       </c>
       <c r="H48" t="s">
-        <v>231</v>
+        <v>221</v>
       </c>
       <c r="I48" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="J48" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="K48" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="L48" t="s">
-        <v>26</v>
+        <v>222</v>
       </c>
       <c r="M48" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="49" spans="1:13" x14ac:dyDescent="0.35">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="49" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>48</v>
       </c>
       <c r="B49" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="C49">
         <v>1</v>
       </c>
+      <c r="D49" t="s">
+        <v>24</v>
+      </c>
       <c r="E49" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="F49" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="G49" t="s">
-        <v>233</v>
+        <v>84</v>
       </c>
       <c r="H49" t="s">
-        <v>104</v>
-      </c>
-      <c r="I49" s="1" t="s">
-        <v>232</v>
+        <v>223</v>
+      </c>
+      <c r="I49" t="s">
+        <v>24</v>
       </c>
       <c r="J49" t="s">
-        <v>234</v>
+        <v>24</v>
       </c>
       <c r="K49" t="s">
-        <v>235</v>
+        <v>24</v>
       </c>
       <c r="L49" t="s">
-        <v>236</v>
+        <v>24</v>
       </c>
       <c r="M49" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="50" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A50">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="50" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A50" s="5">
         <v>49</v>
       </c>
       <c r="B50" t="s">
-        <v>148</v>
+        <v>94</v>
       </c>
       <c r="C50">
         <v>1</v>
       </c>
+      <c r="D50">
+        <v>10</v>
+      </c>
       <c r="E50" t="s">
-        <v>237</v>
+        <v>85</v>
       </c>
       <c r="F50" t="s">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="G50" t="s">
-        <v>241</v>
+        <v>225</v>
       </c>
       <c r="H50" t="s">
-        <v>239</v>
-      </c>
-      <c r="I50" t="s">
-        <v>26</v>
+        <v>101</v>
+      </c>
+      <c r="I50" s="1" t="s">
+        <v>224</v>
       </c>
       <c r="J50" t="s">
-        <v>240</v>
+        <v>226</v>
       </c>
       <c r="K50" t="s">
-        <v>148</v>
+        <v>227</v>
       </c>
       <c r="L50" t="s">
-        <v>238</v>
+        <v>228</v>
       </c>
       <c r="M50" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="51" spans="1:13" x14ac:dyDescent="0.35">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="51" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>50</v>
       </c>
       <c r="B51" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
       <c r="C51">
         <v>1</v>
@@ -3087,38 +3278,111 @@
       <c r="D51">
         <v>4</v>
       </c>
-      <c r="E51" s="1" t="s">
-        <v>242</v>
+      <c r="E51" t="s">
+        <v>229</v>
       </c>
       <c r="F51" t="s">
-        <v>149</v>
+        <v>142</v>
       </c>
       <c r="G51" t="s">
-        <v>243</v>
+        <v>233</v>
       </c>
       <c r="H51" t="s">
-        <v>244</v>
+        <v>231</v>
       </c>
       <c r="I51" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="J51" t="s">
-        <v>26</v>
+        <v>232</v>
       </c>
       <c r="K51" t="s">
-        <v>26</v>
+        <v>140</v>
       </c>
       <c r="L51" t="s">
-        <v>245</v>
+        <v>230</v>
       </c>
       <c r="M51" t="s">
-        <v>80</v>
+        <v>77</v>
+      </c>
+    </row>
+    <row r="52" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A52">
+        <v>51</v>
+      </c>
+      <c r="B52" t="s">
+        <v>139</v>
+      </c>
+      <c r="C52">
+        <v>1</v>
+      </c>
+      <c r="D52">
+        <v>3</v>
+      </c>
+      <c r="E52" s="1" t="s">
+        <v>234</v>
+      </c>
+      <c r="F52" t="s">
+        <v>141</v>
+      </c>
+      <c r="G52" t="s">
+        <v>235</v>
+      </c>
+      <c r="H52" t="s">
+        <v>236</v>
+      </c>
+      <c r="I52" t="s">
+        <v>24</v>
+      </c>
+      <c r="J52" t="s">
+        <v>24</v>
+      </c>
+      <c r="K52" t="s">
+        <v>24</v>
+      </c>
+      <c r="L52" t="s">
+        <v>237</v>
+      </c>
+      <c r="M52" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="53" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A53">
+        <v>52</v>
+      </c>
+      <c r="B53" t="s">
+        <v>24</v>
+      </c>
+      <c r="C53">
+        <v>3</v>
+      </c>
+      <c r="D53">
+        <v>20</v>
+      </c>
+      <c r="E53" t="s">
+        <v>259</v>
+      </c>
+      <c r="F53" t="s">
+        <v>151</v>
+      </c>
+      <c r="G53" t="s">
+        <v>260</v>
+      </c>
+      <c r="H53">
+        <v>603</v>
+      </c>
+      <c r="I53" s="4">
+        <v>0.05</v>
+      </c>
+      <c r="J53" t="s">
+        <v>105</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="E51" numberStoredAsText="1"/>
+    <ignoredError sqref="E21" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>